<commit_message>
fix(ExperienceApp): marking-queue delay (MRKQ) and slow My library load; full run 9 results
- A new submission reaches the teacher's marking queue 4.3-6.6 min after it is made (measured, full run 8):
  TST_MRKQ_TC_1 now waits up to 12 min (step timeout 15 min) and the marking suite (Suite8b) runs after
  Suites 9-14, so most of the delay has passed. Full run 9: MRKQ_TC_1 passed in 2.5 s.
- teacherLibrary.page.js isInitialized waits up to 90 s for the library's search box (it was still loading at
  30 s during the production disruption in full run 9). Not yet verified by a run (user decision).
- Full run 9: 112/113 — MRKQ_TC_1/2 and PROG_TC_1..7 all green; the one failure is TST_TLIB_TC_1 (above).
- Register: MRKQ Pass; TLIB_TC_1 Fail until re-run. Knowledge: marking-queue delay (§A12).

No protected files changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
@@ -927,6 +927,12 @@
     <t>[LP Test Cases] TC_TCH_005. Confirmed live on production 2026-09-23. Module code TLIB agreed with the user 2026-09-23 (teacherLibrary.page.js). Read-only, safe to run repeatedly. The materials view is server-rendered — a click before the page has loaded is ignored (the automation waits for the load).</t>
   </si>
   <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23 (Suite 7 for LP-013/025, Suite 8 for LP-021/022, Suites 9–12 teacher, Suite 13 admin). Full runs 95/96 (learner _6c7t) and 96/96 (teacher _osgr, Class qzwn, learner _xov9) on production — this case passed in both. FAILED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): My library opened but its content was still loading when the 30 s wait ended (production disruption — the same slow teacher-materials request as Add materials). Fix APPLIED 2026-09-24 (the library wait is now ≤ 90 s, user OK) — not yet verified by a run (user: no full run).</t>
+  </si>
+  <si>
     <t>TST_UMBP_TC_11</t>
   </si>
   <si>
@@ -980,7 +986,7 @@
     <t>Confirmed live on production 2026-09-23. The PS counts as completed only once it is evaluated, so 3 (scorable, Flashcards, HTML) of Practice Extra's 4; the PDF is not counted. Page object progress.page.js (module PROG).</t>
   </si>
   <si>
-    <t>Automated 2026-09-23; expected figures moved to the post-marking values 2026-09-24 (Suite 16, last). Debug 9/9 on run 7's users after the Step-1 mark (settled). Earlier: failed in full run 7 on the summary lag — fixed (re-read every 20 s, ≤ 10 min). Full run with marking: NOT yet run (user decision).</t>
+    <t>Automated 2026-09-23/24; post-marking figures. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (the summary figures had settled by the time the check ran).</t>
   </si>
   <si>
     <t>TST_PROG_TC_2</t>
@@ -1006,7 +1012,7 @@
     <t>Confirmed live on production 2026-09-23. Runs at the END of Suite 8, right after the submissions and BEFORE the teacher marks the PS, so the PS row is still pending. Rows are immediate (no lag). Same page as the class card's "See Progress".</t>
   </si>
   <si>
-    <t>Automated 2026-09-23 (passed in full run 7); moved back to the end of Suite 8 on 2026-09-24 (user OK) to check the pending state before marking. Full run with that order: NOT yet run.</t>
+    <t>Automated 2026-09-23; at the end of Suite 8 (pending state before marking). PASSED in full runs 8 and 9 (2026-09-24).</t>
   </si>
   <si>
     <t>TST_PROG_TC_3</t>
@@ -1029,9 +1035,6 @@
   </si>
   <si>
     <t>Confirmed live on production 2026-09-23. The class has one learner, so the class figures follow that learner's.</t>
-  </si>
-  <si>
-    <t>Automated 2026-09-23; post-marking values 2026-09-24 (Suite 15). Debug 9/9 on run 7's users (settled). Summary lag fixed as TC_1. Full run with marking: NOT yet run (user decision).</t>
   </si>
   <si>
     <t>TST_PROG_TC_4</t>
@@ -1057,9 +1060,6 @@
     <t>Confirmed live on production 2026-09-23. Teacher route /class/teacher/…/learner/&lt;id&gt;/bundle/&lt;id&gt;.</t>
   </si>
   <si>
-    <t>Automated 2026-09-23 (passed in full run 7 before marking); post-marking values 2026-09-24. Debug 9/9. Full run with marking: NOT yet run.</t>
-  </si>
-  <si>
     <t>TST_MRKQ_TC_1</t>
   </si>
   <si>
@@ -1085,7 +1085,7 @@
     <t>Confirmed live on production 2026-09-23. MRKQ = markingQueue.page.js. The course/item ids are positional — matched by text. The count can lag the submission (re-read up to 3 min).</t>
   </si>
   <si>
-    <t>Automated 2026-09-24. Grounded by one real mark (user-approved, the same flow) on run 7's data. Cannot be debug-run on marked data — its first automated execution is the next full run (NOT yet run, user decision).</t>
+    <t>Automated 2026-09-24. Full run 8 FAILED: a new submission reaches the queue 4.3–6.6 min after it is made and the step waited only 3 min. Fixed (wait ≤ 12 min; marking suite moved after Suites 9–14). PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (2.5 s — the delay had already passed).</t>
   </si>
   <si>
     <t>TST_MRKQ_TC_2</t>
@@ -1112,6 +1112,9 @@
     <t>Confirmed live on production 2026-09-23. Without feedback the confirmation reads "Send this score without feedback?". MUTATES the run's own data only; the mark cannot be changed afterwards. The Marked tab can lag ("There are no marked student submissions to view" right after).</t>
   </si>
   <si>
+    <t>Automated 2026-09-24. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): marked 70 / "Good", "Ready to send?" confirmed, Unmarked (0).</t>
+  </si>
+  <si>
     <t>TST_PROG_TC_5</t>
   </si>
   <si>
@@ -1132,9 +1135,6 @@
   </si>
   <si>
     <t>Confirmed live on production 2026-09-23. The notification is found by its text (ntf-&lt;n&gt; qids are positional). From SOURCE verifyMarkedPS.</t>
-  </si>
-  <si>
-    <t>Automated 2026-09-24. Grounded by one real mark (user-approved) on run 7's data; debug 9/9 of the marked-state suites. Full run with marking: NOT yet run (user decision).</t>
   </si>
   <si>
     <t>TST_PROG_TC_6</t>
@@ -3858,10 +3858,10 @@
         <v>24</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>25</v>
+        <v>286</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>144</v>
+        <v>287</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -3869,13 +3869,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>17</v>
@@ -3884,19 +3884,19 @@
         <v>18</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>24</v>
@@ -3913,13 +3913,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>17</v>
@@ -3928,19 +3928,19 @@
         <v>18</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>24</v>
@@ -3949,7 +3949,7 @@
         <v>25</v>
       </c>
       <c r="N37" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -3957,13 +3957,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>17</v>
@@ -3972,19 +3972,19 @@
         <v>18</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="L38" s="2" t="s">
         <v>24</v>
@@ -3993,7 +3993,7 @@
         <v>25</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -4001,13 +4001,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>17</v>
@@ -4016,19 +4016,19 @@
         <v>18</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="L39" s="2" t="s">
         <v>24</v>
@@ -4037,7 +4037,7 @@
         <v>25</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -4045,13 +4045,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>17</v>
@@ -4060,19 +4060,19 @@
         <v>18</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L40" s="2" t="s">
         <v>24</v>
@@ -4081,7 +4081,7 @@
         <v>25</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>326</v>
+        <v>304</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -4122,7 +4122,7 @@
         <v>24</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>214</v>
+        <v>25</v>
       </c>
       <c r="N41" s="2" t="s">
         <v>335</v>
@@ -4166,10 +4166,10 @@
         <v>24</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>214</v>
+        <v>25</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -4177,10 +4177,10 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D43" s="2" t="s">
         <v>329</v>
@@ -4192,19 +4192,19 @@
         <v>18</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J43" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>24</v>
@@ -4213,7 +4213,7 @@
         <v>25</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>350</v>
+        <v>304</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -4242,7 +4242,7 @@
         <v>354</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>355</v>
@@ -4257,7 +4257,7 @@
         <v>25</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>350</v>
+        <v>304</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -4301,7 +4301,7 @@
         <v>25</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>350</v>
+        <v>304</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
test(ExperienceApp): Learning Path full runs 10 and 11 both 113/113 — stability confirmed
Two consecutive clean production full runs after the marking-queue and My library
fixes (5b85ebf). Register (.md/.xlsx) execution results, authoring status and the
Learning Path walkthrough updated with the run records.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="602">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="601">
   <si>
     <t>S.No.</t>
   </si>
@@ -927,10 +927,7 @@
     <t>[LP Test Cases] TC_TCH_005. Confirmed live on production 2026-09-23. Module code TLIB agreed with the user 2026-09-23 (teacherLibrary.page.js). Read-only, safe to run repeatedly. The materials view is server-rendered — a click before the page has loaded is ignored (the automation waits for the load).</t>
   </si>
   <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>Automated 2026-09-23 (Suite 7 for LP-013/025, Suite 8 for LP-021/022, Suites 9–12 teacher, Suite 13 admin). Full runs 95/96 (learner _6c7t) and 96/96 (teacher _osgr, Class qzwn, learner _xov9) on production — this case passed in both. FAILED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): My library opened but its content was still loading when the 30 s wait ended (production disruption — the same slow teacher-materials request as Add materials). Fix APPLIED 2026-09-24 (the library wait is now ≤ 90 s, user OK) — not yet verified by a run (user: no full run).</t>
+    <t>Automated 2026-09-23 (Suite 7 for LP-013/025, Suite 8 for LP-021/022, Suites 9–12 teacher, Suite 13 admin). Full runs 95/96 (learner _6c7t) and 96/96 (teacher _osgr, Class qzwn, learner _xov9) on production — this case passed in both. FAILED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): My library opened but its content was still loading when the 30 s wait ended (production disruption — the same slow teacher-materials request as Add materials). Fix APPLIED 2026-09-24 (the library wait is now ≤ 90 s, user OK) — debug run of Suite 12 PASSED 2026-09-24 (8.7 s, teacher _qzro — the library loaded quickly, so the longer wait was not exercised). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y). (the 90 s library wait in place; the library loaded quickly in both).</t>
   </si>
   <si>
     <t>TST_UMBP_TC_11</t>
@@ -986,7 +983,7 @@
     <t>Confirmed live on production 2026-09-23. The PS counts as completed only once it is evaluated, so 3 (scorable, Flashcards, HTML) of Practice Extra's 4; the PDF is not counted. Page object progress.page.js (module PROG).</t>
   </si>
   <si>
-    <t>Automated 2026-09-23/24; post-marking figures. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (the summary figures had settled by the time the check ran).</t>
+    <t>Automated 2026-09-23/24; post-marking figures. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (the summary figures had settled by the time the check ran). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
   </si>
   <si>
     <t>TST_PROG_TC_2</t>
@@ -1012,7 +1009,7 @@
     <t>Confirmed live on production 2026-09-23. Runs at the END of Suite 8, right after the submissions and BEFORE the teacher marks the PS, so the PS row is still pending. Rows are immediate (no lag). Same page as the class card's "See Progress".</t>
   </si>
   <si>
-    <t>Automated 2026-09-23; at the end of Suite 8 (pending state before marking). PASSED in full runs 8 and 9 (2026-09-24).</t>
+    <t>Automated 2026-09-23; at the end of Suite 8 (pending state before marking). PASSED in full runs 8 and 9 (2026-09-24). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
   </si>
   <si>
     <t>TST_PROG_TC_3</t>
@@ -1085,7 +1082,7 @@
     <t>Confirmed live on production 2026-09-23. MRKQ = markingQueue.page.js. The course/item ids are positional — matched by text. The count can lag the submission (re-read up to 3 min).</t>
   </si>
   <si>
-    <t>Automated 2026-09-24. Full run 8 FAILED: a new submission reaches the queue 4.3–6.6 min after it is made and the step waited only 3 min. Fixed (wait ≤ 12 min; marking suite moved after Suites 9–14). PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (2.5 s — the delay had already passed).</t>
+    <t>Automated 2026-09-24. Full run 8 FAILED: a new submission reaches the queue 4.3–6.6 min after it is made and the step waited only 3 min. Fixed (wait ≤ 12 min; marking suite moved after Suites 9–14). PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (2.5 s — the delay had already passed). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
   </si>
   <si>
     <t>TST_MRKQ_TC_2</t>
@@ -1112,7 +1109,7 @@
     <t>Confirmed live on production 2026-09-23. Without feedback the confirmation reads "Send this score without feedback?". MUTATES the run's own data only; the mark cannot be changed afterwards. The Marked tab can lag ("There are no marked student submissions to view" right after).</t>
   </si>
   <si>
-    <t>Automated 2026-09-24. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): marked 70 / "Good", "Ready to send?" confirmed, Unmarked (0).</t>
+    <t>Automated 2026-09-24. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): marked 70 / "Good", "Ready to send?" confirmed, Unmarked (0). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
   </si>
   <si>
     <t>TST_PROG_TC_5</t>
@@ -3858,10 +3855,10 @@
         <v>24</v>
       </c>
       <c r="M35" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N35" s="2" t="s">
         <v>286</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
@@ -3869,34 +3866,34 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G36" s="2" t="s">
+      <c r="H36" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="I36" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="I36" s="2" t="s">
+      <c r="J36" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="J36" s="2" t="s">
+      <c r="K36" s="2" t="s">
         <v>294</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>295</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>24</v>
@@ -3913,43 +3910,43 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="D37" s="2" t="s">
+      <c r="E37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G37" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="E37" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="I37" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="I37" s="2" t="s">
+      <c r="J37" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="J37" s="2" t="s">
+      <c r="K37" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="K37" s="2" t="s">
+      <c r="L37" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N37" s="2" t="s">
         <v>303</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N37" s="2" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
@@ -3957,43 +3954,43 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="I38" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="I38" s="2" t="s">
+      <c r="J38" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="J38" s="2" t="s">
+      <c r="K38" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="K38" s="2" t="s">
+      <c r="L38" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N38" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="L38" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N38" s="2" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
@@ -4001,35 +3998,35 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G39" s="2" t="s">
+      <c r="H39" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="H39" s="2" t="s">
+      <c r="I39" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="I39" s="2" t="s">
+      <c r="J39" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="J39" s="2" t="s">
+      <c r="K39" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="K39" s="2" t="s">
-        <v>319</v>
-      </c>
       <c r="L39" s="2" t="s">
         <v>24</v>
       </c>
@@ -4037,7 +4034,7 @@
         <v>25</v>
       </c>
       <c r="N39" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
@@ -4045,35 +4042,35 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>298</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G40" s="2" t="s">
+      <c r="H40" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="H40" s="2" t="s">
+      <c r="I40" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="I40" s="2" t="s">
+      <c r="J40" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="J40" s="2" t="s">
+      <c r="K40" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="K40" s="2" t="s">
-        <v>326</v>
-      </c>
       <c r="L40" s="2" t="s">
         <v>24</v>
       </c>
@@ -4081,7 +4078,7 @@
         <v>25</v>
       </c>
       <c r="N40" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
@@ -4089,43 +4086,43 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="E41" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G41" s="2" t="s">
+      <c r="H41" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="H41" s="2" t="s">
+      <c r="I41" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="J41" s="2" t="s">
+      <c r="K41" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="K41" s="2" t="s">
+      <c r="L41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N41" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
@@ -4133,43 +4130,43 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="D42" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="D42" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G42" s="2" t="s">
+      <c r="H42" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="H42" s="2" t="s">
+      <c r="I42" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="I42" s="2" t="s">
+      <c r="J42" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="J42" s="2" t="s">
+      <c r="K42" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="K42" s="2" t="s">
+      <c r="L42" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N42" s="2" t="s">
         <v>342</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N42" s="2" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -4177,35 +4174,35 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="C43" s="2" t="s">
+      <c r="D43" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="D43" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="E43" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F43" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G43" s="2" t="s">
+      <c r="H43" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="H43" s="2" t="s">
+      <c r="I43" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="I43" s="2" t="s">
+      <c r="J43" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="J43" s="2" t="s">
+      <c r="K43" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>350</v>
-      </c>
       <c r="L43" s="2" t="s">
         <v>24</v>
       </c>
@@ -4213,7 +4210,7 @@
         <v>25</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
@@ -4221,35 +4218,35 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="C44" s="2" t="s">
+      <c r="D44" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="D44" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G44" s="2" t="s">
+      <c r="H44" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="H44" s="2" t="s">
+      <c r="I44" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="J44" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="I44" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="J44" s="2" t="s">
+      <c r="K44" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="K44" s="2" t="s">
-        <v>356</v>
-      </c>
       <c r="L44" s="2" t="s">
         <v>24</v>
       </c>
@@ -4257,7 +4254,7 @@
         <v>25</v>
       </c>
       <c r="N44" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
@@ -4265,35 +4262,35 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="E45" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F45" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G45" s="2" t="s">
+      <c r="H45" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="I45" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="I45" s="2" t="s">
+      <c r="J45" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="J45" s="2" t="s">
+      <c r="K45" s="2" t="s">
         <v>362</v>
       </c>
-      <c r="K45" s="2" t="s">
-        <v>363</v>
-      </c>
       <c r="L45" s="2" t="s">
         <v>24</v>
       </c>
@@ -4301,7 +4298,7 @@
         <v>25</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -4377,34 +4374,34 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>367</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>368</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J2" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>369</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>370</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>24</v>
@@ -4421,34 +4418,34 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>372</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>373</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>374</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>375</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>24</v>
@@ -4465,34 +4462,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>381</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>382</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>24</v>
@@ -4509,34 +4506,34 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="K5" s="2" t="s">
         <v>388</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>389</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>24</v>
@@ -4553,34 +4550,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>392</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>393</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>394</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>395</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>24</v>
@@ -4597,34 +4594,34 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="K7" s="2" t="s">
         <v>402</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>403</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>24</v>
@@ -4641,34 +4638,34 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>409</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>410</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>24</v>
@@ -4685,34 +4682,34 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>416</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>417</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>24</v>
@@ -4729,34 +4726,34 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="K10" s="2" t="s">
         <v>423</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>424</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>24</v>
@@ -4773,34 +4770,34 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>425</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>426</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>427</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>428</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J11" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="K11" s="2" t="s">
         <v>429</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>430</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>24</v>
@@ -4817,34 +4814,34 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>432</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>433</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>434</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J12" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="K12" s="2" t="s">
         <v>435</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>436</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>24</v>
@@ -4861,34 +4858,34 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>438</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>440</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>441</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>24</v>
@@ -4905,34 +4902,34 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>444</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>445</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>446</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>24</v>
@@ -4949,34 +4946,34 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>447</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>449</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>450</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="I15" s="2" t="s">
         <v>451</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>452</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="K15" s="2" t="s">
         <v>453</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>454</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>24</v>
@@ -4993,34 +4990,34 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>456</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>457</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="I16" s="2" t="s">
         <v>458</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>459</v>
       </c>
-      <c r="J16" s="2" t="s">
-        <v>460</v>
-      </c>
       <c r="K16" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>24</v>
@@ -5037,34 +5034,34 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>461</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>463</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>464</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>465</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J17" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="K17" s="2" t="s">
         <v>466</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>467</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>24</v>
@@ -5081,34 +5078,34 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>467</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>468</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>469</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>470</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>471</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>24</v>
@@ -5125,34 +5122,34 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>474</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>475</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>476</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="J19" s="2" t="s">
         <v>477</v>
       </c>
-      <c r="J19" s="2" t="s">
-        <v>478</v>
-      </c>
       <c r="K19" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>24</v>
@@ -5169,22 +5166,22 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>480</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>481</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>66</v>
@@ -5193,10 +5190,10 @@
         <v>31</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>24</v>
@@ -5213,34 +5210,34 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>483</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>484</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G21" s="2" t="s">
+      <c r="H21" s="2" t="s">
         <v>485</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>486</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>24</v>
@@ -5257,34 +5254,34 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>488</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>489</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>490</v>
       </c>
-      <c r="H22" s="2" t="s">
+      <c r="I22" s="2" t="s">
         <v>491</v>
       </c>
-      <c r="I22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>492</v>
       </c>
-      <c r="J22" s="2" t="s">
-        <v>493</v>
-      </c>
       <c r="K22" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>24</v>
@@ -5301,34 +5298,34 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>494</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="D23" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>495</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>496</v>
       </c>
-      <c r="H23" s="2" t="s">
+      <c r="I23" s="2" t="s">
+        <v>491</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>497</v>
       </c>
-      <c r="I23" s="2" t="s">
-        <v>492</v>
-      </c>
-      <c r="J23" s="2" t="s">
+      <c r="K23" s="2" t="s">
         <v>498</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>499</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>24</v>
@@ -5345,34 +5342,34 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>500</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>501</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G24" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>502</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>503</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>24</v>
@@ -5389,34 +5386,34 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>505</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="D25" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G25" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>507</v>
       </c>
-      <c r="H25" s="2" t="s">
+      <c r="I25" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="2" t="s">
         <v>509</v>
       </c>
-      <c r="J25" s="2" t="s">
+      <c r="K25" s="2" t="s">
         <v>510</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>511</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>24</v>
@@ -5433,34 +5430,34 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>512</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="D26" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>513</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E26" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G26" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>514</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>515</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J26" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="K26" s="2" t="s">
         <v>516</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>517</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>24</v>
@@ -5477,34 +5474,34 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>518</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="D27" s="2" t="s">
+        <v>462</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G27" s="2" t="s">
         <v>519</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>463</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G27" s="2" t="s">
+      <c r="H27" s="2" t="s">
         <v>520</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>521</v>
       </c>
-      <c r="I27" s="2" t="s">
+      <c r="J27" s="2" t="s">
         <v>522</v>
       </c>
-      <c r="J27" s="2" t="s">
+      <c r="K27" s="2" t="s">
         <v>523</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>524</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>24</v>
@@ -5521,34 +5518,34 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>525</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="D28" s="2" t="s">
         <v>526</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="E28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>527</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>528</v>
       </c>
-      <c r="H28" s="2" t="s">
+      <c r="I28" s="2" t="s">
         <v>529</v>
       </c>
-      <c r="I28" s="2" t="s">
+      <c r="J28" s="2" t="s">
         <v>530</v>
       </c>
-      <c r="J28" s="2" t="s">
-        <v>531</v>
-      </c>
       <c r="K28" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>24</v>
@@ -5565,34 +5562,34 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>532</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="D29" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>533</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" s="2" t="s">
+      <c r="H29" s="2" t="s">
         <v>534</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>535</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>24</v>
@@ -5609,34 +5606,34 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>537</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="D30" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>538</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" s="2" t="s">
+      <c r="H30" s="2" t="s">
         <v>539</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>540</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>24</v>
@@ -5653,34 +5650,34 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>541</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>542</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="D31" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>543</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>544</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>545</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L31" s="2" t="s">
         <v>24</v>
@@ -5697,22 +5694,22 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>547</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="D32" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G32" s="2" t="s">
         <v>548</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>549</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>66</v>
@@ -5721,10 +5718,10 @@
         <v>31</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>24</v>
@@ -5741,34 +5738,34 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>550</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>551</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="D33" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>552</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G33" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>553</v>
       </c>
-      <c r="H33" s="2" t="s">
+      <c r="I33" s="2" t="s">
         <v>554</v>
       </c>
-      <c r="I33" s="2" t="s">
+      <c r="J33" s="2" t="s">
         <v>555</v>
       </c>
-      <c r="J33" s="2" t="s">
-        <v>556</v>
-      </c>
       <c r="K33" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>24</v>
@@ -5785,34 +5782,34 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>556</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>557</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="D34" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>558</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>559</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>24</v>
@@ -5829,34 +5826,34 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>560</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>561</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="D35" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>562</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>527</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G35" s="2" t="s">
+      <c r="H35" s="2" t="s">
         <v>563</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="I35" s="2" t="s">
+        <v>554</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>564</v>
       </c>
-      <c r="I35" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="J35" s="2" t="s">
+      <c r="K35" s="2" t="s">
         <v>565</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>566</v>
       </c>
       <c r="L35" s="2" t="s">
         <v>24</v>
@@ -5873,34 +5870,34 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>567</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="D36" s="2" t="s">
         <v>568</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="E36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="E36" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G36" s="2" t="s">
+      <c r="H36" s="2" t="s">
         <v>570</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>571</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J36" s="2" t="s">
+        <v>571</v>
+      </c>
+      <c r="K36" s="2" t="s">
         <v>572</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>573</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>24</v>
@@ -5917,34 +5914,34 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>574</v>
       </c>
-      <c r="C37" s="2" t="s">
+      <c r="D37" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G37" s="2" t="s">
         <v>575</v>
       </c>
-      <c r="D37" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>576</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>577</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J37" s="2" t="s">
+        <v>577</v>
+      </c>
+      <c r="K37" s="2" t="s">
         <v>578</v>
-      </c>
-      <c r="K37" s="2" t="s">
-        <v>579</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>24</v>
@@ -5961,34 +5958,34 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>579</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>580</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="D38" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>581</v>
       </c>
-      <c r="D38" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G38" s="2" t="s">
+      <c r="H38" s="2" t="s">
         <v>582</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="I38" s="2" t="s">
+        <v>529</v>
+      </c>
+      <c r="J38" s="2" t="s">
         <v>583</v>
       </c>
-      <c r="I38" s="2" t="s">
-        <v>530</v>
-      </c>
-      <c r="J38" s="2" t="s">
+      <c r="K38" s="2" t="s">
         <v>584</v>
-      </c>
-      <c r="K38" s="2" t="s">
-        <v>585</v>
       </c>
       <c r="L38" s="2" t="s">
         <v>24</v>
@@ -6005,34 +6002,34 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>586</v>
       </c>
-      <c r="C39" s="2" t="s">
+      <c r="D39" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="2" t="s">
         <v>587</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G39" s="2" t="s">
+      <c r="H39" s="2" t="s">
         <v>588</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>589</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L39" s="2" t="s">
         <v>24</v>
@@ -6049,34 +6046,34 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>590</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>591</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>592</v>
       </c>
-      <c r="D40" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G40" s="2" t="s">
+      <c r="H40" s="2" t="s">
         <v>593</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>594</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="L40" s="2" t="s">
         <v>24</v>
@@ -6093,34 +6090,34 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>596</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>597</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>569</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G41" s="2" t="s">
+      <c r="H41" s="2" t="s">
         <v>598</v>
       </c>
-      <c r="H41" s="2" t="s">
+      <c r="I41" s="2" t="s">
         <v>599</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
         <v>600</v>
       </c>
-      <c r="J41" s="2" t="s">
-        <v>601</v>
-      </c>
       <c r="K41" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
feat(tooling): stakeholder summary report + Learning Path automation (#73)
Stakeholder summary report built after every run (ADR-024; renumbered from ADR-023 on merge because main already has ADR-023 for the eBook/FOC consolidation), full-page end-of-test screenshots, and Learning Path production automation. Mochawesome report unchanged.
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="601">
   <si>
     <t>S.No.</t>
   </si>
@@ -285,19 +285,22 @@
     <t>#LP-007 — Drilling into a unit from the open TOC sidebar reveals that unit's activity list</t>
   </si>
   <si>
-    <t>Learner (with an activated product and a joined class) is inside Practice Extra, on the Learning Path unit view. The TOC sidebar is open (TST_PEXT_TC_2).</t>
-  </si>
-  <si>
-    <t>1. Click a unit-level item in the TOC (div.unit-level-item).</t>
-  </si>
-  <si>
-    <t>The unit's individual activities (e.g. the non-scorable and PS entries) become visible and selectable in the TOC card.</t>
-  </si>
-  <si>
-    <t>From SOURCE playwright-automation-c1 (live-verified by that team); confirm live when automating. Matches LearningpathPage.goInsideUnit(). Precondition for LP-008 and LP-010.</t>
-  </si>
-  <si>
-    <t>Not Run</t>
+    <t>Learner (with an activated product and a joined class) is inside Practice Extra, on the Learning Path unit view. The TOC sidebar is open at its UNIT view (housekeeping TST_PEXT_TC_101 — the open control lands on the lesson view on every entry but the first).</t>
+  </si>
+  <si>
+    <t>1. Click the unit row "Unit 1" in the TOC unit view (.unit-level-item).</t>
+  </si>
+  <si>
+    <t>Unit "Unit 1"; activities of cqaautomationbundle1: BASE04_Dropdown_Scorable.zip, Flashcards.zip, PS, Non-scorable HTML activity, test pdf</t>
+  </si>
+  <si>
+    <t>The TOC switches to the unit's lesson view (header "Unit 1", "Lesson 1" expanded) and lists all five activities; the unit list is no longer shown.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Matches SOURCE LearningpathPage.goInsideUnit(). Precondition for LP-008 and LP-010.</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23 in learningPath.json Suite 8 (Suite 6 for DASH_TC_15). Debug run 21/21 (learner _uyu7); full runs 74/75 (learner _vcmw) and 75/75 (learner _iyit) — this case passed in both.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_10</t>
@@ -318,10 +321,10 @@
     <t>Activity: "Flashcards.zip" (product cqaautomationbundle1)</t>
   </si>
   <si>
-    <t>The non-scorable activity's iframe content (the flashcard deck) loads.</t>
-  </si>
-  <si>
-    <t>From SOURCE playwright-automation-c1 (live-verified by that team); confirm live when automating. Matches LearningpathPage.openNonScorable().</t>
+    <t>The player's activity title reads "Flashcards.zip" and the flashcard deck (6 cards, step bar) loads in the activity iframe. The TOC stays open.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Matches SOURCE LearningpathPage.openNonScorable().</t>
   </si>
   <si>
     <t>TST_PEXT_TC_11</t>
@@ -336,16 +339,17 @@
     <t>The Flashcards activity has just loaded (TST_PEXT_TC_10).</t>
   </si>
   <si>
-    <t>1. Click "Next" to advance the deck, waiting for each card to render, until the deck ends.</t>
-  </si>
-  <si>
-    <t>SOURCE uses a fixed 5 clicks for this deck — see LP-017 for the risk in that assumption.</t>
-  </si>
-  <si>
-    <t>Each click advances the flashcard deck and no check/grade control is offered at any point (the activity is non-scorable).</t>
-  </si>
-  <si>
-    <t>From SOURCE playwright-automation-c1 (live-verified by that team); confirm live when automating. Prefer driving the loop from the deck's own state (last-card signal) rather than a hardcoded 5 — see LP-017.</t>
+    <t xml:space="preserve">1. If the deck is not on its first card, go back with "Previous" (the deck remembers where the learner left it).
+2. Click "Next" once per card, waiting for the card to change, until the last card is current.</t>
+  </si>
+  <si>
+    <t>Deck of 6 cards (cqaautomationbundle1). No fixed click count — the loop follows the deck's step bar (LP-017).</t>
+  </si>
+  <si>
+    <t>Each Next advances exactly one card, from the first to the last (6 of 6); on the last card the bar offers "Previous" and "NEXT ACTIVITY". No Check / grading control is offered at any point.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. A Next clicked within ~1.8 s of the previous card change is ignored (≥ 2.0 s always accepted) — the automation waits 2.5 s per card. Clicking "NEXT ACTIVITY" moves on to the PS.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_12</t>
@@ -366,10 +370,10 @@
     <t>Activity: "PS"</t>
   </si>
   <si>
-    <t>The PS free-text rich-editor answer screen is shown.</t>
-  </si>
-  <si>
-    <t>From SOURCE playwright-automation-c1 (live-verified by that team); confirm live when automating. Matches LearningpathPage.openPS().</t>
+    <t>The player's activity title reads "PS" and the free-text answer screen is shown: instructions, an "Answer:" rich editor ("Type here …", B/I/U, "Word count: 0"), Save and Submit.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. The PS is NOT inside the activity iframe (outer page). Matches SOURCE LearningpathPage.openPS().</t>
   </si>
   <si>
     <t>TST_PEXT_TC_13</t>
@@ -392,10 +396,10 @@
     <t>Answer text: "Submitting PS activity"</t>
   </si>
   <si>
-    <t>The "attempted answer" confirmation (div.attempted-answer) is shown, confirming the submission was accepted.</t>
-  </si>
-  <si>
-    <t>From SOURCE playwright-automation-c1 (live-verified by that team); confirm live when automating. Matches LearningpathPage.submitPS(). PS is free text and NOT auto-graded — the answer enters the teacher's marking queue (marking itself belongs to the class area, not here). ONE ATTEMPT PER LEARNER: plan the run like the scorable activity.</t>
+    <t>Typing enables Submit; Submit opens "Ready to submit?" ("…it won't be possible to make any changes to your work after it's submitted", Cancel / Submit); confirming closes it and the answer is shown read-only (div.attempted-answer = the typed text). The editor and Submit are gone; the TOC marks PS "evaluation pending".</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Matches SOURCE LearningpathPage.submitPS(). PS is free text and NOT auto-graded — the answer enters the teacher's marking queue. ONE ATTEMPT PER LEARNER: plan the run like the scorable activity.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_14</t>
@@ -432,7 +436,7 @@
     <t>TST_PEXT_TC_15</t>
   </si>
   <si>
-    <t>Verify what happens when check is clicked on a scorable frame with no option selected</t>
+    <t>Verify Check is not offered on a scorable frame until a dropdown option is chosen</t>
   </si>
   <si>
     <t>#LP-013 — Clicking check on a scorable frame without selecting any dropdown option</t>
@@ -441,16 +445,23 @@
     <t>Negative</t>
   </si>
   <si>
-    <t>Learner is on a scorable activity frame; no dropdown opened or selected.</t>
-  </si>
-  <si>
-    <t>1. Without opening or selecting any option, click the green check button.</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Inferred: the check is rejected / no-ops, or an explicit empty-answer state is shown.</t>
-  </si>
-  <si>
-    <t>Not exercised by SOURCE (it always selects an answer first). Capture the real copy when confirming, and keep it out of the same run as the happy-path scorable case (one attempt per learner).</t>
+    <t>Learner is on frame 1 of the scorable activity; no dropdown opened or selected (first attempt).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Without opening or selecting any option, look for the green Check button.
+2. Choose an option (TST_PEXT_TC_4).</t>
+  </si>
+  <si>
+    <t>Frame 1 (0-based 0)</t>
+  </si>
+  <si>
+    <t>With nothing chosen, NO Check button is shown, so an empty check cannot be made; Check appears once an option is chosen (TST_PEXT_TC_4).</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. (fresh learner _5an7). Fits the sheet's inferred "rejected / no-op". It consumes nothing, so it runs inside the learner's one scorable attempt in Suite 7, just before TST_PEXT_TC_4 — no second learner needed (user question 2026-09-23).</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23 (Suite 7 for LP-013/025, Suite 8 for LP-021/022, Suites 9–12 teacher, Suite 13 admin). Full runs 95/96 (learner _6c7t) and 96/96 (teacher _osgr, Class qzwn, learner _xov9) on production — this case passed in both.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_16</t>
@@ -469,10 +480,10 @@
 2. Click the submit-answer button.</t>
   </si>
   <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Inferred: submission is blocked (e.g. a validation message), since PS expects a free-text response.</t>
-  </si>
-  <si>
-    <t>Not exercised by SOURCE (it always types an answer first).</t>
+    <t>Submit is disabled while the editor is empty ("Word count: 0"): it is greyed out, clicking it opens no "Ready to submit?" dialog and nothing is submitted. No validation message is shown.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Submit is disabled by CSS class only (class="btn disabled", no disabled attribute). Safe to run before TST_PEXT_TC_13 — it does not consume the learner's one PS submission. Not exercised by SOURCE.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_17</t>
@@ -490,20 +501,23 @@
     <t>The learner has already submitted a PS answer for this activity.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Navigate away from the PS activity (e.g. via the TOC).
-2. Navigate back into the same PS activity.</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Inferred: the "attempted answer" indicator shows immediately on re-entry and the editor / submit controls are no longer offered for a fresh submission.</t>
-  </si>
-  <si>
-    <t>Natural follow-on from LP-011 in the same run, since the PS is already submitted by then.</t>
+    <t xml:space="preserve">1. Open another activity from the TOC (Flashcards.zip).
+2. Open the PS again from the TOC.</t>
+  </si>
+  <si>
+    <t>Away: "Flashcards.zip"; back: "PS"</t>
+  </si>
+  <si>
+    <t>The submitted answer is shown read-only (the text that was submitted); there is no editor and no Submit, so no fresh submission is possible.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Natural follow-on from LP-011 in the same run, since the PS is already submitted by then.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_18</t>
   </si>
   <si>
-    <t>Verify the learner leaves the Learning Path when the lesson-view panel is closed</t>
+    <t>Verify closing the lesson-view panel closes the TOC and keeps the learner in the Learning Path</t>
   </si>
   <si>
     <t>#LP-018 — Closing the main lesson-view panel returns the learner out of the Learning Path view</t>
@@ -512,22 +526,40 @@
     <t>Low</t>
   </si>
   <si>
-    <t>Learner is within a unit/activity view inside the Learning Path.</t>
-  </si>
-  <si>
-    <t>1. Click the lesson-view close control (#lessonViewCrossBtn).</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Inferred: the learner returns to the class dashboard or the previous screen.</t>
-  </si>
-  <si>
-    <t>SOURCE has closeMainSideBar() but never calls it — dead code there, so treat it as unverified. Note our own TOC close control is a different element (see LP-006 / learning-path-player.md).</t>
+    <t>Learner is inside the Learning Path with the TOC open on its lesson view.</t>
+  </si>
+  <si>
+    <t>1. Click the lesson-view close control (✕, #lessonViewCrossBtn).</t>
+  </si>
+  <si>
+    <t>The TOC closes; the learner stays in the Learning Path on the same activity (it does NOT leave the player). Leaving is done with the player's "Back" link — see TST_PEXT_TC_26.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. The scenario sheet assumed this control left the Learning Path; on production it only closes the TOC. SOURCE's closeMainSideBar() was dead code.</t>
+  </si>
+  <si>
+    <t>TST_PEXT_TC_26</t>
+  </si>
+  <si>
+    <t>Verify the player's Back link returns the learner from the Learning Path to the dashboard</t>
+  </si>
+  <si>
+    <t>Learner is inside the Learning Path (any activity), TOC closed.</t>
+  </si>
+  <si>
+    <t>1. Click "Back" (top left of the player).</t>
+  </si>
+  <si>
+    <t>The learner is returned to the learner dashboard (/dashboard/learner/dashboard).</t>
+  </si>
+  <si>
+    <t>APPENDED 2026-09-23 while automating LP-018: the scenario's intent ("return the learner out of the Learning Path view") is met by Back, not by the lesson-view close control. Confirmed live on production 2026-09-23.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_19</t>
   </si>
   <si>
-    <t>Verify the TOC sidebar stays in one consistent open state when the open control is clicked again</t>
+    <t>Verify the TOC sidebar stays in one consistent state when the open control is activated again while open</t>
   </si>
   <si>
     <t>#LP-019 — Opening the TOC sidebar a second time without closing it first</t>
@@ -536,13 +568,14 @@
     <t>The TOC sidebar is already open.</t>
   </si>
   <si>
-    <t>1. With the sidebar open, click the open-sidebar control again.</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Inferred: the sidebar remains in a single consistent open state (no duplicate panel, no corrupted layout).</t>
-  </si>
-  <si>
-    <t>While the TOC is open it covers the open-sidebar control on production (2026-09-22) — reaching this state may itself need a scroll or a different entry point; record what is found.</t>
+    <t xml:space="preserve">1. With the sidebar open, move keyboard focus to the open-sidebar control (the activity title link) and press Enter.
+2. Press Enter again.</t>
+  </si>
+  <si>
+    <t>The control is a toggle: the first Enter CLOSES the TOC, the second re-opens it. There is never more than one sidebar and the layout stays intact.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. While the TOC is open it covers the open control, so a mouse cannot click it again — only the keyboard can. The sheet assumed the TOC would simply stay open; it toggles instead (a consistent state, not a defect — flagged to the product owner to confirm).</t>
   </si>
   <si>
     <t>TST_DASH_TC_15</t>
@@ -557,68 +590,72 @@
     <t>A learner who has signed up and verified but has NOT joined a class or activated a product.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Log in as that learner.
-2. Look for a "Practice Extra" entry point on the dashboard.</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Inferred: the "Practice Extra" entry point is absent (or disabled) until a product is activated and a class joined.</t>
-  </si>
-  <si>
-    <t>Cheap to run in the LP suite: the run's learner is in exactly this state between TST_SNUP_TC_64 (verified) and the invite being accepted.</t>
+    <t xml:space="preserve">1. Log in as that learner (who has a pending class invite).
+2. Look for a class card and a "Practice Extra" entry point.</t>
+  </si>
+  <si>
+    <t>Class of the LP run (invited, not accepted); component "Practice Extra"</t>
+  </si>
+  <si>
+    <t>The learner is NOT shown the dashboard: login routes straight to the "Invitations (1)" page, listing the invited class (Accept disabled until it is ticked). No class card and no "Practice Extra" entry point are shown.</t>
+  </si>
+  <si>
+    <t>Runs in the LP suite's Suite 6, after the learner logs in and BEFORE the invite is accepted (between TST_SNUP_TC_64 and TST_INVI_TC_4) — so only a full run exercises it; a --runData=last learner already has the class.</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23 (Suite 6). First full run (learner _vcmw) failed on the test design — it expected the dashboard, but a learner with a pending invite is routed to the Invitations page; fixed, then full run 75/75 (learner _iyit) passed.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_20</t>
   </si>
   <si>
-    <t>Verify an HTML activity completes by itself after a short dwell</t>
+    <t>Verify an HTML activity completes by itself (no submit) and counts toward the unit completion</t>
   </si>
   <si>
     <t>#LP-021 — Learner launches an HTML activity within a PE component (auto-completes after a dwell)</t>
   </si>
   <si>
-    <t>A PE component containing an HTML activity; learner has access.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Log in as the learner.
-2. Launch the PE component.
-3. Navigate to the HTML activity.
-4. Wait about 3 seconds without interacting.</t>
-  </si>
-  <si>
-    <t>The HTML activity loads without error and is marked completed after the dwell, with no explicit submit.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_LRN_002. No page-object support in SOURCE; selectors must be captured live.</t>
-  </si>
-  <si>
-    <t>BLOCKED: needs a product whose PE component contains an HTML activity — cqaautomationbundle1 (the suite's product) has Scorable, Flashcards, PS and Projects only. Unblock = such a product on the test school.</t>
+    <t>Learner inside Practice Extra, TOC open on the lesson view of Unit 1; the HTML activity not yet opened.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Note the unit's completion counter in the TOC unit view ("N/4 Completed").
+2. Open Unit 1 and open "Non-scorable HTML activity".
+3. Wait a few seconds without interacting.
+4. Check the activity's TOC status and the unit counter again.</t>
+  </si>
+  <si>
+    <t>Unit 1; activity "Non-scorable HTML activity"</t>
+  </si>
+  <si>
+    <t>The HTML activity loads in the player; within seconds its TOC status becomes "Activity status: viewed" with no submit, and the unit counter goes up by one (e.g. 2/4 → 3/4 Completed).</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_LRN_002. Confirmed live on production 2026-09-23. "viewed" is the completed state of a non-scorable activity (it counts in "N/4 Completed"); reached ~1.5 s after opening (the sheet said a ~3 s dwell). Was wrongly Blocked at design time (the product does have an HTML activity).</t>
   </si>
   <si>
     <t>TST_PEXT_TC_21</t>
   </si>
   <si>
-    <t>Verify a PDF activity completes by itself after a short dwell</t>
+    <t>Verify a downloadable PDF activity is marked viewed when the learner lands on it, with no download or submit</t>
   </si>
   <si>
     <t>#LP-022 — Learner launches a PDF activity within a PE component (auto-completes after a dwell)</t>
   </si>
   <si>
-    <t>A PE component containing a PDF activity; learner has access.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Log in as the learner.
-2. Launch the PE component.
-3. Navigate to the PDF activity.
-4. Wait about 3 seconds without interacting.</t>
-  </si>
-  <si>
-    <t>The PDF activity loads without error and is marked completed after the dwell, with no explicit submit.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_LRN_002. No page-object support in SOURCE.</t>
-  </si>
-  <si>
-    <t>BLOCKED: needs a product whose PE component contains a PDF activity (see TST_PEXT_TC_20).</t>
+    <t>Learner on the HTML activity (TST_PEXT_TC_20); the PDF activity "test pdf" not yet visited.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click NEXT ACTIVITY in the player.
+2. Look at the page and at the activity's TOC status. Do NOT click Download.</t>
+  </si>
+  <si>
+    <t>Activity "test pdf" (file Sample1.pdf)</t>
+  </si>
+  <si>
+    <t>The player lands on "test pdf" and shows a DOWNLOAD page — "Download the test pdf below and complete this activity", the file name "Sample1.pdf" and a Download button (the PDF itself is not displayed and nothing is downloaded). Landing on it marks the activity "Activity status: viewed", with no submit.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_LRN_002. Confirmed live on production 2026-09-23. The TOC marks it "Downloadable item". Landing on it (e.g. via NEXT ACTIVITY after the HTML activity) is what marks it viewed — confirmed as expected by the user 2026-09-23. The suite never clicks Download.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_22</t>
@@ -647,7 +684,10 @@
     <t>[LP Test Cases] TC_LRN_003. Multi-actor (2 learners + teacher) — plan the run accordingly.</t>
   </si>
   <si>
-    <t>BLOCKED: needs a group-enabled component with a Collab activity, 2 learners and a class group. Class groups are not automated yet (planned as a separate module). Unblock = that product/data plus group creation.</t>
+    <t>Not Run</t>
+  </si>
+  <si>
+    <t>ON HOLD — user 2026-09-23: do not automate until confirmed. The design-time blockers are resolved: the group-enabled (NLP) component is Projects (cqaautomationpr1) with "Collaborative Task" and "Group PS"; groups are created from Class data → Students/Groups toggle → "+ Create groups" (user screenshot); a second learner per run is approved for these two cases only (parked setup: learningPathGroups.json, verified 65/65). Plan agreed: modules NLPP / CGRP / MRKQ; mark 90, comment "Well Done".</t>
   </si>
   <si>
     <t>TST_PEXT_TC_23</t>
@@ -674,7 +714,7 @@
     <t>[LP Test Cases] TC_LRN_003. Depends on marking + analytics, which are separate un-migrated areas.</t>
   </si>
   <si>
-    <t>BLOCKED: as TST_PEXT_TC_22, plus the teacher marking queue and analytics are not automated yet.</t>
+    <t>ON HOLD — user 2026-09-23: as TST_PEXT_TC_22. Teacher marks in the marking queue with score 90 and comment "Well Done" (user decision).</t>
   </si>
   <si>
     <t>TST_PEXT_TC_24</t>
@@ -686,22 +726,24 @@
     <t>#LP-025 — Exiting a Scorable activity before submitting saves it in a "Saved" in-progress state</t>
   </si>
   <si>
-    <t>A PE component with a scorable activity the learner has NOT completed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Log in as the learner and open Practice Extra → a unit → a lesson.
-2. Launch the scorable activity and answer part of it without completing.
-3. Exit back to the TOC.
-4. Relaunch the same activity.</t>
-  </si>
-  <si>
-    <t>Use the same answers as TST_PEXT_TC_4 (frame 1) — stop before the final Next.</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Inferred from the sheet: the TOC shows the activity as "Saved" (in progress), not complete/scored, and relaunching restores the answers already entered.</t>
-  </si>
-  <si>
-    <t>Needs a learner whose scorable activity is untouched — mutually exclusive with LP-002/003 in the same run (one attempt per learner). Plan a dedicated learner, or run this INSTEAD of the full scorable pass.</t>
+    <t>Frame 1 of the scorable activity has been answered and checked (TST_PEXT_TC_4); frames 2–4 not yet done.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the TOC and open another activity (Flashcards.zip).
+2. Look at the scorable activity's status in the TOC.
+3. Open the scorable activity again from the TOC.</t>
+  </si>
+  <si>
+    <t>Scorable: BASE04_Dropdown_Scorable.zip; away: Flashcards.zip</t>
+  </si>
+  <si>
+    <t>While away, the TOC shows the scorable as "Activity status: in progress" (not completed, no score). Reopening it lands on the frame where the learner left it, with the checked answer kept (still marked correct) and Next offered, so the attempt continues (frames 2–4 then score 4 out of 4).</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. (fresh learner _5an7). The sheet's "Saved" = re-landing on the same screen where the learner left it; the TOC label is "in progress" (user, 2026-09-23 — wording, not a defect). Runs inside the learner's one attempt in Suite 7, right after TST_PEXT_TC_4.</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23 (Suite 7, between TST_PEXT_TC_4 and TC_5). First full run (learner _6c7t) failed on the test: on a FIRST entry the TOC reopens on the unit view, which lists no activities — fixed by opening it on the lesson view first; full run 96/96 (learner _xov9) passed. Flashcards is only where the learner navigates to; the saved state checked is the scorable's.</t>
   </si>
   <si>
     <t>TST_PEXT_TC_25</t>
@@ -716,23 +758,25 @@
     <t>A PE/LP component whose TOC has units containing lessons containing activities.</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Log in as the learner and open Practice Extra.
-2. Expand a unit node, then a lesson node under it.
-3. Collapse the lesson node, then the unit node.
-4. Open an activity, then click "Back".
-5. Click "Back" again to return to unit level.</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. Each node expands/collapses and keeps its state; "Back" returns activity → lesson → unit without losing context, and the right children render at each level.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_LRN_005. Deeper than LP-005/006/007. Check whether cqaautomationbundle1's TOC actually has three levels; if it does not, this needs another product and becomes Blocked.</t>
+    <t xml:space="preserve">1. With the TOC on the lesson view of "Unit 1" (after TST_PEXT_TC_9), click the "Lesson 1" heading to collapse it.
+2. Click it again to expand it.
+3. Click "Go to unit view" (‹ in the TOC).
+4. Click "Unit 1" again.</t>
+  </si>
+  <si>
+    <t>Unit "Unit 1", lesson "Lesson 1", the five activities of TST_PEXT_TC_9</t>
+  </si>
+  <si>
+    <t>Collapsing hides the lesson's activities and expanding shows them again; "Go to unit view" replaces the lesson view with the unit list; opening "Unit 1" again returns to the same lesson with the same five activities.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_LRN_005. Confirmed live on production 2026-09-23. cqaautomationbundle1 has three levels (Unit 1 &gt; Lesson 1 &gt; activities). Units do not collapse in place — a unit opens its own lesson view, and "Go to unit view" is the level-up ("Back") control. Opening an activity keeps the TOC on the same lesson view.</t>
   </si>
   <si>
     <t>TST_DASH_TC_16</t>
   </si>
   <si>
-    <t>Verify an SLE-activated component shows no expiry date and a progress bar while it loads</t>
+    <t>Verify an SLE-activated component shows no expiry date and a loading indicator while it launches</t>
   </si>
   <si>
     <t>#LP-027 — An SLE-activated PE/LP component shows no expiry date and a progress bar on launch</t>
@@ -750,10 +794,10 @@
     <t>Class of the LP run; component "Practice Extra"</t>
   </si>
   <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. No expiry date under the SLE-activated component; launching shows a progress bar before the Learning Path content renders.</t>
-  </si>
-  <si>
-    <t>The SLE half is already proven by TST_DASH_TC_13 (tile present, no activation-code prompt). This case adds the expiry-date absence and the loading progress bar. Watch the false-green trap: ".progress-container" is the permanent "See Progress" card, not the loading bar.</t>
+    <t>No expiry date on the SLE-activated component (the tile reads "Practice Extra / Continue learning"; the class card shows only the class start → end dates). Launching shows a loading SPINNER for about a second, then the Learning Path player opens.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. The sheet expected a PROGRESS BAR; production shows a spinner (div.loader, ~0.2–1.1 s after the click) — no progress bar was observed (flagged to the product owner). The SLE half is already proven by TST_DASH_TC_13. False-green trap: ".progress-container" is the permanent "See Progress" card.</t>
   </si>
   <si>
     <t>TST_CMAT_TC_7</t>
@@ -774,13 +818,13 @@
 4. Expand the product and click the Practice Extra component.</t>
   </si>
   <si>
-    <t>Class of the LP run; product cqaautomationbundle1</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. The component launches for the teacher and its TOC renders, so the teacher can preview activities without submitting.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_TCH_001. Module CMAT (classMaterials.page.js) already exists for the Materials tab; the LP launch from it is new. Teacher preview must not create learner progress — confirm.</t>
+    <t>Class of the LP run; product cqaautomationbundle1; component "Practice Extra"</t>
+  </si>
+  <si>
+    <t>The Materials tab lists the product's components (Practice Extra, Projects, Test, Showcase); clicking Practice Extra opens the Learning Path on the teacher route (/learning-path/teacher/…) with an activity loaded and its TOC rendered (unit view, "Unit 1"), for preview.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_TCH_001. Confirmed live on production 2026-09-23. The TOC opens by itself only on the user's first entry — on later entries the test opens it with the player's control. A teacher preview does NOT create learner progress (confirmed by the user 2026-09-23; not asserted by the test).</t>
   </si>
   <si>
     <t>TST_C1AS_TC_26</t>
@@ -795,16 +839,13 @@
     <t xml:space="preserve">1. Log in as the teacher and open the class.
 2. Open the "Assignments" tab.
 3. Click "Create assignment".
-4. Select and launch the LP component inside the flow.</t>
-  </si>
-  <si>
-    <t>Class of the LP run</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. The LP component launches for the teacher and its TOC renders inside assignment creation.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_TCH_002. Module C1AS (c1assignment) covers assignments today; check its existing TCs before adding selectors.</t>
+4. Click "Practice Extra" in the component list. Do NOT click Next / Assign.</t>
+  </si>
+  <si>
+    <t>Create assignment lists the product's components (Practice Extra, Projects, Test); clicking Practice Extra opens the Learning Path in assignment mode (/learning-path/teacher/…/assignments/…) with its TOC ("Practice Extra", unit "Unit 1") and Cancel / Next. No assignment is created.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_TCH_002. Confirmed live on production 2026-09-23. Launch only — the user decided nothing is saved (2026-09-23); the component is addressed by name (its qid a-path-2-&lt;n&gt; is positional).</t>
   </si>
   <si>
     <t>TST_C1AS_TC_27</t>
@@ -825,13 +866,13 @@
 4. Select and launch the NLP component.</t>
   </si>
   <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. The component launches in the LP app/view and its TOC renders.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_TCH_003. The sheet marks the whole scenario an ASSUMPTION — confirm with product/design that NLP appears here at all.</t>
-  </si>
-  <si>
-    <t>BLOCKED: NLP/Projects is not automated anywhere yet, and the sheet flags the scenario itself as unverified. Unblock = confirm the flow exists, then automate after the NLP player.</t>
+    <t>Create assignment lists Projects; clicking it opens the Learning Path in assignment mode (/learning-path/teacher/…/assignments/product/cqaautomationpr1/…) with its TOC (unit "Unit 1") and Cancel / Next. No assignment is created.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_TCH_003. Confirmed live on production 2026-09-23. The NLP component is Projects (cqaautomationpr1); the flow exists (was Blocked as unverified). Launch only, like TST_C1AS_TC_26 (Suite 14).</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23 (learningPath.json Suite 14). Debug 3/3; passed in full run 7 on 2026-09-24 (103/105; teacher _4n9d, Class u62l, learner _yqma).</t>
   </si>
   <si>
     <t>TST_MSAC_TC_1</t>
@@ -847,14 +888,15 @@
   </si>
   <si>
     <t xml:space="preserve">1. Log in as the teacher and open the class.
-2. Open the "Materials" tab and click "Manage student access".
-3. Start creating a lock/unlock rule and launch the LP component from that flow.</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. The LP component launches for the teacher and its TOC renders.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_TCH_004. Module code MSAC is PROPOSED — no page object exists for "Manage student access"; agree the code when the page object is created (AGENTS.md Rule 6). Creating a lock rule changes class state — decide before running whether the rule is removed afterwards (ADR-021).</t>
+2. Open the "Materials" tab and click the product's "Manage student access".
+3. Click "Create access rule".
+4. Click "Practice Extra" in the component list. Do NOT click Continue.</t>
+  </si>
+  <si>
+    <t>"Manage student access" opens with "Create access rule"; the rule flow lists the product's components; clicking Practice Extra opens the Learning Path in rule-creation mode (/learning-path/teacher/…/create-access) with its TOC ("Select all units", unit checkboxes) and Cancel / Continue. No rule is created.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_TCH_004. Confirmed live on production 2026-09-23. Module code MSAC agreed with the user 2026-09-23 (manageStudentAccess.page.js). Launch only — Continue is never clicked, so class state is unchanged (user decision 2026-09-23). The visible "Select all units" control is the checkbox wrapper; its &lt;label&gt; is screen-reader-only.</t>
   </si>
   <si>
     <t>TST_TLIB_TC_1</t>
@@ -870,22 +912,25 @@
   </si>
   <si>
     <t xml:space="preserve">1. Log in as the teacher.
-2. Open the "My library" tab on the teacher dashboard.
-3. Find/search the product.
-4. Open the product ("View details" / bundle view).
-5. Launch the Practice Extra component.</t>
-  </si>
-  <si>
-    <t>Product cqaautomationbundle1</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. The component launches for the teacher and its TOC renders.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_TCH_005. Module code TLIB is PROPOSED — no page object exists for the teacher "My library" tab. Read-only case, safe to run repeatedly.</t>
-  </si>
-  <si>
-    <t>TST_UMBP_TC_5</t>
+2. Open "My library" on the teacher dashboard.
+3. Search the product (Enter).
+4. Click the product title (expands its card), then "View details".
+5. Click "Practice Extra".</t>
+  </si>
+  <si>
+    <t>Product cqaautomationbundle1; component "Practice Extra"</t>
+  </si>
+  <si>
+    <t>My library (/dashboard/teacher/library) finds the product; its card expands with its components and "View details"; View details opens the product materials view (/dashboard/teacher/…/bundle/cqaautomationbundle1/view); Practice Extra opens the Learning Path on the teacher route with its TOC rendered.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_TCH_005. Confirmed live on production 2026-09-23. Module code TLIB agreed with the user 2026-09-23 (teacherLibrary.page.js). Read-only, safe to run repeatedly. The materials view is server-rendered — a click before the page has loaded is ignored (the automation waits for the load).</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23 (Suite 7 for LP-013/025, Suite 8 for LP-021/022, Suites 9–12 teacher, Suite 13 admin). Full runs 95/96 (learner _6c7t) and 96/96 (teacher _osgr, Class qzwn, learner _xov9) on production — this case passed in both. FAILED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): My library opened but its content was still loading when the 30 s wait ended (production disruption — the same slow teacher-materials request as Add materials). Fix APPLIED 2026-09-24 (the library wait is now ≤ 90 s, user OK) — debug run of Suite 12 PASSED 2026-09-24 (8.7 s, teacher _qzro — the library loaded quickly, so the longer wait was not exercised). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y). (the 90 s library wait in place; the library loaded quickly in both).</t>
+  </si>
+  <si>
+    <t>TST_UMBP_TC_11</t>
   </si>
   <si>
     <t>Verify an admin can launch an LP component from the Library tab's product materials</t>
@@ -894,23 +939,241 @@
     <t>#LP-033 — Admin launches an LP component under an umbrella product via the Library tab</t>
   </si>
   <si>
-    <t>School-admin login; the school library contains an umbrella product with an LP component.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Log in as the admin.
+    <t>School-admin login (prod_admin_mqa@yopmail.com, single-school admin of MQA Sierra School MQA-ABC-DEF); the school library contains the product.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Log in as the admin (lands straight in the school).
 2. Open the "LIBRARY" tab.
 3. Search the product.
-4. Click "See materials".
-5. Launch the LP component.</t>
-  </si>
-  <si>
-    <t>An umbrella product on the admin's school (e.g. the SLE product of the LP school)</t>
-  </si>
-  <si>
-    <t>[ASSUMED] The scenario sheet states this behaviour is not confirmed — verify live before automating. The Library tab shows "School licence" and "All course materials"; search filters to matching products; "See materials" opens the component list; the LP component launches for preview and renders.</t>
-  </si>
-  <si>
-    <t>[LP Test Cases] TC_ADM_001. Module UMBP (umbrellaProduct — product materials view) already covers "See materials"; only the LP launch is new. The Library tab itself is covered by LIBR in AdminApp-Library — check that register for overlap before automating.</t>
+4. Click its row ("See materials").
+5. Click "Practice Extra".</t>
+  </si>
+  <si>
+    <t>Product cqaautomationbundle1; component "Practice Extra"; school key MQA-ABC-DEF</t>
+  </si>
+  <si>
+    <t>The Library tab shows the School licence section and the product list; the search lists the product; "See materials" opens the product materials view (components Practice Extra, Projects, Test); Practice Extra opens the Learning Path preview on the teacher route with its TOC rendered.</t>
+  </si>
+  <si>
+    <t>[LP Test Cases] TC_ADM_001. Confirmed live on production 2026-09-23. RENAMED from TST_UMBP_TC_5 (that id is retired in AdminApp-Library) with the user's OK. The sheet's "All course materials" heading belongs to the teacher's My library, not the admin Library tab — dropped (user, 2026-09-23). The materials view is server-rendered: clicks before its document has loaded are ignored (measured) — the automation waits for the load.</t>
+  </si>
+  <si>
+    <t>TST_PROG_TC_1</t>
+  </si>
+  <si>
+    <t>Verify the learner My progress counts the submitted activities overall and per component</t>
+  </si>
+  <si>
+    <t>#LP-034 — Learner and teacher progress views reflect the learner's submitted activities (added on user request 2026-09-23 — not in lp-scenarios.xlsx)</t>
+  </si>
+  <si>
+    <t>The learner has, in this run, completed the scorable activity (4/4), paged Flashcards, submitted the PS (not yet marked) and viewed the HTML activity and the PDF (Suites 7–8). Learner on the dashboard.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. On the class card, click "My progress".
+2. Read the summary and the Practice Extra / Projects blocks.</t>
+  </si>
+  <si>
+    <t>Class of the LP run; components Practice Extra, Projects</t>
+  </si>
+  <si>
+    <t>"My progress" shows, once the batch job has updated it (minutes after the mark): Completed activities 4/10, Activities completed above target score 2/4, 85% Average score. Practice Extra: 4/4, above target 2/4, below target 0/4, 85%. Projects: 0/5. (after the teacher marked the PS 70 / "Good", Suite 8b) Before marking the same page showed 3/10 · 1/3 · 100% (the PS is not counted until evaluated).</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. The PS counts as completed only once it is evaluated, so 3 (scorable, Flashcards, HTML) of Practice Extra's 4; the PDF is not counted. Page object progress.page.js (module PROG).</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23/24; post-marking figures. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (the summary figures had settled by the time the check ran). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
+  </si>
+  <si>
+    <t>TST_PROG_TC_2</t>
+  </si>
+  <si>
+    <t>Verify the learner per-activity progress shows each submitted activity's result</t>
+  </si>
+  <si>
+    <t>Learner on "My progress" (TST_PROG_TC_1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click the product card (cqaautomationbundle1).
+2. Click "Practice Extra".
+3. Read the Unit 1 / Lesson 1 activity rows.</t>
+  </si>
+  <si>
+    <t>Product cqaautomationbundle1; component Practice Extra</t>
+  </si>
+  <si>
+    <t>Rows: BASE04_Dropdown_Scorable.zip — First score 100%, Best score 100%, Attempts 1, icon "Completed above target"; Flashcards.zip — Viewed ("Activity status: viewed"); PS — First score -, Best score -, Attempts 1 ("Activity status: evaluation pending"); Non-scorable HTML activity — Viewed; test pdf — Viewed.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Runs at the END of Suite 8, right after the submissions and BEFORE the teacher marks the PS, so the PS row is still pending. Rows are immediate (no lag). Same page as the class card's "See Progress".</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-23; at the end of Suite 8 (pending state before marking). PASSED in full runs 8 and 9 (2026-09-24). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
+  </si>
+  <si>
+    <t>TST_PROG_TC_3</t>
+  </si>
+  <si>
+    <t>Verify the teacher Class data shows the class and learner figures for the submitted activities</t>
+  </si>
+  <si>
+    <t>The learner has, in this run, completed the scorable activity (4/4), paged Flashcards, submitted the PS (not yet marked) and viewed the HTML activity and the PDF (Suites 7–8). Teacher on the class page (Class data tab).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the class from the teacher dashboard (Class data is the default tab).
+2. Read Class performance and the learner's card.</t>
+  </si>
+  <si>
+    <t>Class of the LP run; learner "Learner User"</t>
+  </si>
+  <si>
+    <t>Class data (once updated): Average completed activities 40%, Activities completed above target score 2 /4, 85% Average score; the learner's card 4/10, 2/4, 85%. (after the teacher marked the PS 70 / "Good", Suite 8b) Before marking: 30% · 1 /3 · 100% and 3/10.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. The class has one learner, so the class figures follow that learner's.</t>
+  </si>
+  <si>
+    <t>TST_PROG_TC_4</t>
+  </si>
+  <si>
+    <t>Verify the teacher per-activity view of a learner matches the learner's own progress</t>
+  </si>
+  <si>
+    <t>Teacher on Class data (TST_PROG_TC_3).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click the learner's product link (cqaautomationbundle1).
+2. Click "Practice Extra".
+3. Read the activity rows.</t>
+  </si>
+  <si>
+    <t>Learner "Learner User"; product cqaautomationbundle1; component Practice Extra</t>
+  </si>
+  <si>
+    <t>The teacher sees the same rows as the learner: scorable 100% / 100% / 1 attempt; Flashcards / HTML / PDF Viewed; PS First score 70%, Best score 70%, Attempts 1 ("Completed above target") (after the teacher marked the PS 70 / "Good", Suite 8b).</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Teacher route /class/teacher/…/learner/&lt;id&gt;/bundle/&lt;id&gt;.</t>
+  </si>
+  <si>
+    <t>TST_MRKQ_TC_1</t>
+  </si>
+  <si>
+    <t>Verify the marking queue lists the learner's Practice Set submission with the score pre-filled</t>
+  </si>
+  <si>
+    <t>#LP-035 — Teacher marks the learner's Practice Set; the mark reaches the learner and the progress at both ends (added on user request 2026-09-24, from SOURCE ClassDashboardPage)</t>
+  </si>
+  <si>
+    <t>The learner has submitted the PS (TST_PEXT_TC_13); teacher on the class page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Look at the class's "Marking" link.
+2. Open it; open "Practice Extra", then "Unit 1: Lesson 1 / PS", then the learner's submission.</t>
+  </si>
+  <si>
+    <t>Course Practice Extra; item "Unit 1: Lesson 1 / PS"; learner "Learner User"</t>
+  </si>
+  <si>
+    <t>The class shows "1 Marking" (the dashboard card a badge 1). The queue shows "Unmarked (1)", "Practice Extra (1) cqaautomationbundle1", "Unit 1: Lesson 1 / PS" and the learner's submission; the marking screen shows the answer "Submitting PS activity", Score % pre-filled with 70, a Feedback editor, Save and Send.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. MRKQ = markingQueue.page.js. The course/item ids are positional — matched by text. The count can lag the submission (re-read up to 3 min).</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-24. Full run 8 FAILED: a new submission reaches the queue 4.3–6.6 min after it is made and the step waited only 3 min. Fixed (wait ≤ 12 min; marking suite moved after Suites 9–14). PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b) (2.5 s — the delay had already passed). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
+  </si>
+  <si>
+    <t>TST_MRKQ_TC_2</t>
+  </si>
+  <si>
+    <t>Verify a Practice Set is marked when the teacher sends a score and feedback and confirms it</t>
+  </si>
+  <si>
+    <t>The learner's PS is open on the marking screen (TST_MRKQ_TC_1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Set Score to 70.
+2. Type the feedback "Good".
+3. Click Send.
+4. Confirm with Send in "Ready to send?".</t>
+  </si>
+  <si>
+    <t>Score 70 (SOURCE's value — pre-filled); feedback "Good" (user decision 2026-09-24)</t>
+  </si>
+  <si>
+    <t>"Ready to send? Once sent, you won't be able to make any further changes" opens; after Send the queue shows "Unmarked (0)", the item "70% … Marked", the submission "Score : 70 %" and the teacher block "Score: 70 % Feedback: Good".</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Without feedback the confirmation reads "Send this score without feedback?". MUTATES the run's own data only; the mark cannot be changed afterwards. The Marked tab can lag ("There are no marked student submissions to view" right after).</t>
+  </si>
+  <si>
+    <t>Automated 2026-09-24. PASSED in full run 9 on 2026-09-24 (112/113; teacher _qzro, Class e6tb, learner _m10b): marked 70 / "Good", "Ready to send?" confirmed, Unmarked (0). Two consecutive clean full runs on 2026-09-24: run 10 113/113 (teacher _z959, Class kgk8, learner _e78s) and run 11 113/113 (teacher _8sw6, Class htbu, learner _wf0y).</t>
+  </si>
+  <si>
+    <t>TST_PROG_TC_5</t>
+  </si>
+  <si>
+    <t>Verify the learner receives the teacher's feedback notification with the mark</t>
+  </si>
+  <si>
+    <t>The teacher has marked the run's learner's PS (TST_MRKQ_TC_2, Suite 8b). Learner logged in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the notifications bell.
+2. Click "New feedback".</t>
+  </si>
+  <si>
+    <t>Score 70; feedback "Good"</t>
+  </si>
+  <si>
+    <t>The bell lists "New feedback · PS · Your teacher has sent you some feedback"; it opens the PS in the player showing "Score : 70 %" and the teacher's "Score: 70 % Feedback: Good".</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. The notification is found by its text (ntf-&lt;n&gt; qids are positional). From SOURCE verifyMarkedPS.</t>
+  </si>
+  <si>
+    <t>TST_PROG_TC_6</t>
+  </si>
+  <si>
+    <t>Verify the learner's per-activity progress shows the marked Practice Set's score</t>
+  </si>
+  <si>
+    <t>The teacher has marked the run's learner's PS (TST_MRKQ_TC_2, Suite 8b). Learner on "My progress" (TST_PROG_TC_1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click the product card.
+2. Click "Practice Extra".
+3. Read the PS row.</t>
+  </si>
+  <si>
+    <t>PS: First score 70%, Best score 70%, Attempts 1, icon "Completed above target"; the lesson reads 4/4 Completed, 85%. The other rows are unchanged.</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. Rows update immediately after the mark (only the summary totals lag).</t>
+  </si>
+  <si>
+    <t>TST_PROG_TC_7</t>
+  </si>
+  <si>
+    <t>Verify the teacher's progress details show the learner's per-component figures after marking</t>
+  </si>
+  <si>
+    <t>The teacher has marked the run's learner's PS (TST_MRKQ_TC_2, Suite 8b). Teacher on Class data.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Switch on "Show progress details".
+2. Read the learner's Practice Extra and Projects blocks.</t>
+  </si>
+  <si>
+    <t>Learner "Learner User"</t>
+  </si>
+  <si>
+    <t>Practice Extra: Completed activities 4/4, above target 2/4, below target 0/4, 85%. Projects: Completed activities 0/5 (0 Gold medals, "-" average). Test: "This student has not activated the code yet".</t>
+  </si>
+  <si>
+    <t>Confirmed live on production 2026-09-23. The switch's checkbox is visually hidden — its label is clicked. From SOURCE toggleProgressBar / verifyTeacherAnalyticsBundleLevel.</t>
   </si>
   <si>
     <t>TST_LAND_TC_2</t>
@@ -2042,7 +2305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2524,22 +2787,22 @@
         <v>88</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
@@ -2547,13 +2810,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>17</v>
@@ -2562,28 +2825,28 @@
         <v>72</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
@@ -2591,13 +2854,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>17</v>
@@ -2606,28 +2869,28 @@
         <v>72</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -2635,13 +2898,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>17</v>
@@ -2650,28 +2913,28 @@
         <v>18</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
@@ -2679,13 +2942,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>17</v>
@@ -2694,28 +2957,28 @@
         <v>18</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
@@ -2723,13 +2986,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>17</v>
@@ -2738,28 +3001,28 @@
         <v>18</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
@@ -2767,43 +3030,43 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>31</v>
+        <v>141</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>24</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -2811,43 +3074,43 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M18" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
@@ -2855,43 +3118,43 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>72</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>31</v>
+        <v>158</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
@@ -2899,43 +3162,43 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
@@ -2943,43 +3206,43 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>152</v>
+        <v>17</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N21" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -2987,43 +3250,43 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>137</v>
+        <v>155</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>72</v>
+        <v>164</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
@@ -3031,43 +3294,43 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>17</v>
+        <v>138</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>31</v>
+        <v>187</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>132</v>
+        <v>25</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
@@ -3075,13 +3338,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>17</v>
@@ -3090,28 +3353,28 @@
         <v>18</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>31</v>
+        <v>196</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>132</v>
+        <v>25</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>194</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
@@ -3119,13 +3382,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>17</v>
@@ -3134,28 +3397,28 @@
         <v>18</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>31</v>
+        <v>204</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>132</v>
+        <v>25</v>
       </c>
       <c r="N25" s="2" t="s">
-        <v>202</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
@@ -3163,13 +3426,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>17</v>
@@ -3178,28 +3441,28 @@
         <v>18</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>132</v>
+        <v>214</v>
       </c>
       <c r="N26" s="2" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
@@ -3207,43 +3470,43 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="G27" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M27" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="H27" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="N27" s="2" t="s">
-        <v>24</v>
+        <v>223</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
@@ -3251,13 +3514,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>17</v>
@@ -3266,28 +3529,28 @@
         <v>72</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>31</v>
+        <v>229</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>24</v>
+        <v>232</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
@@ -3295,43 +3558,43 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M29" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N29" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
@@ -3339,13 +3602,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>17</v>
@@ -3354,28 +3617,28 @@
         <v>18</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M30" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>24</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
@@ -3383,13 +3646,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>17</v>
@@ -3398,28 +3661,28 @@
         <v>18</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="L31" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M31" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N31" s="2" t="s">
-        <v>24</v>
+        <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
@@ -3427,13 +3690,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>17</v>
@@ -3445,25 +3708,25 @@
         <v>252</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>31</v>
+        <v>246</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>132</v>
+        <v>25</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>256</v>
+        <v>144</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
@@ -3471,13 +3734,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>17</v>
@@ -3486,28 +3749,28 @@
         <v>18</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>246</v>
+        <v>31</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>24</v>
+        <v>270</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
@@ -3515,13 +3778,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>17</v>
@@ -3530,28 +3793,28 @@
         <v>18</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>269</v>
+        <v>254</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>24</v>
+        <v>144</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -3559,13 +3822,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>17</v>
@@ -3574,28 +3837,468 @@
         <v>18</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="L35" s="2" t="s">
         <v>24</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>91</v>
+        <v>25</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>24</v>
+        <v>286</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="L43" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M43" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="L44" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M44" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="L45" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M45" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -3671,13 +4374,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>280</v>
+        <v>363</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>281</v>
+        <v>364</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>282</v>
+        <v>365</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>17</v>
@@ -3686,19 +4389,19 @@
         <v>18</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>283</v>
+        <v>366</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>284</v>
+        <v>367</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>285</v>
+        <v>368</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>286</v>
+        <v>369</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>24</v>
@@ -3715,13 +4418,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>287</v>
+        <v>370</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>288</v>
+        <v>371</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>282</v>
+        <v>365</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>17</v>
@@ -3730,19 +4433,19 @@
         <v>18</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>283</v>
+        <v>366</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>289</v>
+        <v>372</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>290</v>
+        <v>373</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>291</v>
+        <v>374</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>24</v>
@@ -3759,13 +4462,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>292</v>
+        <v>375</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>293</v>
+        <v>376</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>282</v>
+        <v>365</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>17</v>
@@ -3774,19 +4477,19 @@
         <v>18</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>294</v>
+        <v>377</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>295</v>
+        <v>378</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>296</v>
+        <v>379</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>297</v>
+        <v>380</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>298</v>
+        <v>381</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>24</v>
@@ -3803,13 +4506,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>299</v>
+        <v>382</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>300</v>
+        <v>383</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>282</v>
+        <v>365</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>17</v>
@@ -3818,19 +4521,19 @@
         <v>18</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>301</v>
+        <v>384</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>302</v>
+        <v>385</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>303</v>
+        <v>386</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>304</v>
+        <v>387</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>24</v>
@@ -3847,13 +4550,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>306</v>
+        <v>389</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>307</v>
+        <v>390</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>282</v>
+        <v>365</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>17</v>
@@ -3862,19 +4565,19 @@
         <v>18</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>308</v>
+        <v>391</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>309</v>
+        <v>392</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>310</v>
+        <v>393</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>311</v>
+        <v>394</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>24</v>
@@ -3891,13 +4594,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>312</v>
+        <v>395</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>313</v>
+        <v>396</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>314</v>
+        <v>397</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>17</v>
@@ -3906,19 +4609,19 @@
         <v>18</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>315</v>
+        <v>398</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>316</v>
+        <v>399</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>317</v>
+        <v>400</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>318</v>
+        <v>401</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>319</v>
+        <v>402</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>24</v>
@@ -3935,13 +4638,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>320</v>
+        <v>403</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>321</v>
+        <v>404</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>314</v>
+        <v>397</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>17</v>
@@ -3950,19 +4653,19 @@
         <v>18</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>322</v>
+        <v>405</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>323</v>
+        <v>406</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>324</v>
+        <v>407</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>325</v>
+        <v>408</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>326</v>
+        <v>409</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>24</v>
@@ -3979,13 +4682,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>327</v>
+        <v>410</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>328</v>
+        <v>411</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>314</v>
+        <v>397</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>17</v>
@@ -3994,19 +4697,19 @@
         <v>18</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>329</v>
+        <v>412</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>330</v>
+        <v>413</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>331</v>
+        <v>414</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>332</v>
+        <v>415</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>333</v>
+        <v>416</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>24</v>
@@ -4023,13 +4726,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>334</v>
+        <v>417</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>335</v>
+        <v>418</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>314</v>
+        <v>397</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>17</v>
@@ -4038,19 +4741,19 @@
         <v>18</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>336</v>
+        <v>419</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>337</v>
+        <v>420</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>338</v>
+        <v>421</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>339</v>
+        <v>422</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>340</v>
+        <v>423</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>24</v>
@@ -4067,13 +4770,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>341</v>
+        <v>424</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>342</v>
+        <v>425</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>314</v>
+        <v>397</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>17</v>
@@ -4082,19 +4785,19 @@
         <v>18</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>343</v>
+        <v>426</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>344</v>
+        <v>427</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>345</v>
+        <v>428</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>346</v>
+        <v>429</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>24</v>
@@ -4111,13 +4814,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>347</v>
+        <v>430</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>348</v>
+        <v>431</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>314</v>
+        <v>397</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>17</v>
@@ -4126,19 +4829,19 @@
         <v>18</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>349</v>
+        <v>432</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>350</v>
+        <v>433</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>351</v>
+        <v>434</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>352</v>
+        <v>435</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>24</v>
@@ -4155,13 +4858,13 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>353</v>
+        <v>436</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>354</v>
+        <v>437</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>355</v>
+        <v>438</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>17</v>
@@ -4170,19 +4873,19 @@
         <v>18</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>356</v>
+        <v>439</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>357</v>
+        <v>440</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>358</v>
+        <v>441</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>352</v>
+        <v>435</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>24</v>
@@ -4199,13 +4902,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>359</v>
+        <v>442</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>360</v>
+        <v>443</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>355</v>
+        <v>438</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>17</v>
@@ -4214,19 +4917,19 @@
         <v>18</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>361</v>
+        <v>444</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>362</v>
+        <v>445</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>363</v>
+        <v>446</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>352</v>
+        <v>435</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>24</v>
@@ -4243,13 +4946,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>364</v>
+        <v>447</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>365</v>
+        <v>448</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>355</v>
+        <v>438</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>17</v>
@@ -4258,19 +4961,19 @@
         <v>18</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>366</v>
+        <v>449</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>367</v>
+        <v>450</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>368</v>
+        <v>451</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>369</v>
+        <v>452</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>370</v>
+        <v>453</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>24</v>
@@ -4287,13 +4990,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>371</v>
+        <v>454</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>372</v>
+        <v>455</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>355</v>
+        <v>438</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>17</v>
@@ -4302,19 +5005,19 @@
         <v>18</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>373</v>
+        <v>456</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>374</v>
+        <v>457</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>375</v>
+        <v>458</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>376</v>
+        <v>459</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>352</v>
+        <v>435</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>24</v>
@@ -4331,13 +5034,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>377</v>
+        <v>460</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>378</v>
+        <v>461</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>17</v>
@@ -4346,19 +5049,19 @@
         <v>18</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>380</v>
+        <v>463</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>381</v>
+        <v>464</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>382</v>
+        <v>465</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>383</v>
+        <v>466</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>24</v>
@@ -4375,13 +5078,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>384</v>
+        <v>467</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>385</v>
+        <v>468</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>17</v>
@@ -4390,19 +5093,19 @@
         <v>18</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>386</v>
+        <v>469</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>387</v>
+        <v>470</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J18" s="2" t="s">
+        <v>471</v>
+      </c>
+      <c r="K18" s="2" t="s">
         <v>388</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>305</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>24</v>
@@ -4419,13 +5122,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>389</v>
+        <v>472</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>390</v>
+        <v>473</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>17</v>
@@ -4434,19 +5137,19 @@
         <v>18</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>391</v>
+        <v>474</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>392</v>
+        <v>475</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>393</v>
+        <v>476</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>394</v>
+        <v>477</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>24</v>
@@ -4463,13 +5166,13 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>395</v>
+        <v>478</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>396</v>
+        <v>479</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>17</v>
@@ -4478,7 +5181,7 @@
         <v>18</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>397</v>
+        <v>480</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>66</v>
@@ -4487,10 +5190,10 @@
         <v>31</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>398</v>
+        <v>481</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>24</v>
@@ -4507,13 +5210,13 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>399</v>
+        <v>482</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>400</v>
+        <v>483</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>17</v>
@@ -4522,19 +5225,19 @@
         <v>18</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>401</v>
+        <v>484</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>402</v>
+        <v>485</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>403</v>
+        <v>486</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>24</v>
@@ -4551,13 +5254,13 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>404</v>
+        <v>487</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>405</v>
+        <v>488</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>17</v>
@@ -4566,19 +5269,19 @@
         <v>18</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>406</v>
+        <v>489</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>407</v>
+        <v>490</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>408</v>
+        <v>491</v>
       </c>
       <c r="J22" s="2" t="s">
-        <v>409</v>
+        <v>492</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>24</v>
@@ -4595,13 +5298,13 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>410</v>
+        <v>493</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>411</v>
+        <v>494</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>17</v>
@@ -4610,19 +5313,19 @@
         <v>18</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>412</v>
+        <v>495</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>413</v>
+        <v>496</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>408</v>
+        <v>491</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>414</v>
+        <v>497</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>415</v>
+        <v>498</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>24</v>
@@ -4639,13 +5342,13 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>416</v>
+        <v>499</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>417</v>
+        <v>500</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>17</v>
@@ -4654,19 +5357,19 @@
         <v>18</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>418</v>
+        <v>501</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>419</v>
+        <v>502</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>420</v>
+        <v>503</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>24</v>
@@ -4683,13 +5386,13 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>421</v>
+        <v>504</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>422</v>
+        <v>505</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>17</v>
@@ -4698,19 +5401,19 @@
         <v>18</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>423</v>
+        <v>506</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>424</v>
+        <v>507</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>425</v>
+        <v>508</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>426</v>
+        <v>509</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>427</v>
+        <v>510</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>24</v>
@@ -4727,13 +5430,13 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>428</v>
+        <v>511</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>429</v>
+        <v>512</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>17</v>
@@ -4742,19 +5445,19 @@
         <v>18</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>430</v>
+        <v>513</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>431</v>
+        <v>514</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>432</v>
+        <v>515</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>433</v>
+        <v>516</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>24</v>
@@ -4771,13 +5474,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>434</v>
+        <v>517</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>435</v>
+        <v>518</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>379</v>
+        <v>462</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>17</v>
@@ -4786,19 +5489,19 @@
         <v>18</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>436</v>
+        <v>519</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>437</v>
+        <v>520</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>438</v>
+        <v>521</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>439</v>
+        <v>522</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>440</v>
+        <v>523</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>24</v>
@@ -4815,13 +5518,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>441</v>
+        <v>524</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>442</v>
+        <v>525</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>17</v>
@@ -4830,19 +5533,19 @@
         <v>18</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>444</v>
+        <v>527</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>445</v>
+        <v>528</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>446</v>
+        <v>529</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>447</v>
+        <v>530</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>24</v>
@@ -4859,13 +5562,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>448</v>
+        <v>531</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>449</v>
+        <v>532</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>17</v>
@@ -4874,19 +5577,19 @@
         <v>18</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>450</v>
+        <v>533</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>451</v>
+        <v>534</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>452</v>
+        <v>535</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>24</v>
@@ -4903,13 +5606,13 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>453</v>
+        <v>536</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>454</v>
+        <v>537</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>17</v>
@@ -4918,19 +5621,19 @@
         <v>18</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>455</v>
+        <v>538</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>456</v>
+        <v>539</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>457</v>
+        <v>540</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>24</v>
@@ -4947,13 +5650,13 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>458</v>
+        <v>541</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>459</v>
+        <v>542</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>17</v>
@@ -4962,19 +5665,19 @@
         <v>18</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>460</v>
+        <v>543</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>461</v>
+        <v>544</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>462</v>
+        <v>545</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L31" s="2" t="s">
         <v>24</v>
@@ -4991,13 +5694,13 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>463</v>
+        <v>546</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>464</v>
+        <v>547</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>17</v>
@@ -5006,7 +5709,7 @@
         <v>18</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>465</v>
+        <v>548</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>66</v>
@@ -5015,10 +5718,10 @@
         <v>31</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>466</v>
+        <v>549</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>24</v>
@@ -5035,13 +5738,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>467</v>
+        <v>550</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>468</v>
+        <v>551</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>17</v>
@@ -5050,19 +5753,19 @@
         <v>18</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>469</v>
+        <v>552</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>470</v>
+        <v>553</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>471</v>
+        <v>554</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>472</v>
+        <v>555</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>24</v>
@@ -5079,13 +5782,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>473</v>
+        <v>556</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>474</v>
+        <v>557</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>17</v>
@@ -5094,19 +5797,19 @@
         <v>18</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>301</v>
+        <v>384</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>475</v>
+        <v>558</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>476</v>
+        <v>559</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>24</v>
@@ -5123,13 +5826,13 @@
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>477</v>
+        <v>560</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>478</v>
+        <v>561</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>443</v>
+        <v>526</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>17</v>
@@ -5138,19 +5841,19 @@
         <v>18</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>479</v>
+        <v>562</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>480</v>
+        <v>563</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>471</v>
+        <v>554</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>481</v>
+        <v>564</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>482</v>
+        <v>565</v>
       </c>
       <c r="L35" s="2" t="s">
         <v>24</v>
@@ -5167,13 +5870,13 @@
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>483</v>
+        <v>566</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>484</v>
+        <v>567</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>485</v>
+        <v>568</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>17</v>
@@ -5182,19 +5885,19 @@
         <v>18</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>486</v>
+        <v>569</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>487</v>
+        <v>570</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>488</v>
+        <v>571</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>489</v>
+        <v>572</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>24</v>
@@ -5211,13 +5914,13 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>490</v>
+        <v>573</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>491</v>
+        <v>574</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>485</v>
+        <v>568</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>17</v>
@@ -5226,19 +5929,19 @@
         <v>18</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>492</v>
+        <v>575</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>493</v>
+        <v>576</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>494</v>
+        <v>577</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>495</v>
+        <v>578</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>24</v>
@@ -5255,13 +5958,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>496</v>
+        <v>579</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>497</v>
+        <v>580</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>485</v>
+        <v>568</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>17</v>
@@ -5270,19 +5973,19 @@
         <v>18</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>498</v>
+        <v>581</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>499</v>
+        <v>582</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>446</v>
+        <v>529</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>500</v>
+        <v>583</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>501</v>
+        <v>584</v>
       </c>
       <c r="L38" s="2" t="s">
         <v>24</v>
@@ -5299,13 +6002,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>502</v>
+        <v>585</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>503</v>
+        <v>586</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>485</v>
+        <v>568</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>17</v>
@@ -5314,19 +6017,19 @@
         <v>18</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>504</v>
+        <v>587</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>505</v>
+        <v>588</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>506</v>
+        <v>589</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L39" s="2" t="s">
         <v>24</v>
@@ -5343,13 +6046,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>507</v>
+        <v>590</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>508</v>
+        <v>591</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>485</v>
+        <v>568</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>17</v>
@@ -5358,19 +6061,19 @@
         <v>18</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>509</v>
+        <v>592</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>510</v>
+        <v>593</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>31</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>511</v>
+        <v>594</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>305</v>
+        <v>388</v>
       </c>
       <c r="L40" s="2" t="s">
         <v>24</v>
@@ -5387,13 +6090,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>512</v>
+        <v>595</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>513</v>
+        <v>596</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>485</v>
+        <v>568</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>17</v>
@@ -5402,19 +6105,19 @@
         <v>18</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>514</v>
+        <v>597</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>515</v>
+        <v>598</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>516</v>
+        <v>599</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>517</v>
+        <v>600</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>352</v>
+        <v>435</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
fix(ExperienceApp): LP progress totals after the Projects product update
Projects gained its HTML + PDF activities on 2026-09-25, so the learner's
overall total went /10 -> /11 and Projects /5 -> /6. The LP suite still
expected the old figures and failed 3 progress checks on production
(TST_PROG_TC_1/3/7; 110/113).

- learningPathData.json (progressMarked): 4/10 -> 4/11, 40% -> 36%,
  Projects 0/5 -> 0/6
- learning-path-player.md: totals updated, note on bundle-content changes
- LP register: three expected results updated (regenerated .md/.xlsx)
- authoring-status.md index line + walkthrough session 8

Verified on production: learningPathTest_prod 113/113 (407 checks) twice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
+++ b/testAutomation_v1.0/test/Manual/C1App/LearningPath/LearningPath_test_cases.xlsx
@@ -977,7 +977,7 @@
     <t>Class of the LP run; components Practice Extra, Projects</t>
   </si>
   <si>
-    <t>"My progress" shows, once the batch job has updated it (minutes after the mark): Completed activities 4/10, Activities completed above target score 2/4, 85% Average score. Practice Extra: 4/4, above target 2/4, below target 0/4, 85%. Projects: 0/5. (after the teacher marked the PS 70 / "Good", Suite 8b) Before marking the same page showed 3/10 · 1/3 · 100% (the PS is not counted until evaluated).</t>
+    <t>"My progress" shows, once the batch job has updated it (minutes after the mark): Completed activities 4/11, Activities completed above target score 2/4, 85% Average score. Practice Extra: 4/4, above target 2/4, below target 0/4, 85%. Projects: 0/6. (after the teacher marked the PS 70 / "Good", Suite 8b) Before marking the same page showed 3/11 · 1/3 · 100% (the PS is not counted until evaluated). [2026-09-29] Totals updated after the Projects update (HTML + PDF added 2026-09-25): /10 → /11, Projects /5 → /6.</t>
   </si>
   <si>
     <t>Confirmed live on production 2026-09-23. The PS counts as completed only once it is evaluated, so 3 (scorable, Flashcards, HTML) of Practice Extra's 4; the PDF is not counted. Page object progress.page.js (module PROG).</t>
@@ -1028,7 +1028,7 @@
     <t>Class of the LP run; learner "Learner User"</t>
   </si>
   <si>
-    <t>Class data (once updated): Average completed activities 40%, Activities completed above target score 2 /4, 85% Average score; the learner's card 4/10, 2/4, 85%. (after the teacher marked the PS 70 / "Good", Suite 8b) Before marking: 30% · 1 /3 · 100% and 3/10.</t>
+    <t>Class data (once updated): Average completed activities 36%, Activities completed above target score 2 /4, 85% Average score; the learner's card 4/11, 2/4, 85%. (after the teacher marked the PS 70 / "Good", Suite 8b) Before marking: 27% · 1 /3 · 100% and 3/11. [2026-09-29] Was 40% / 4/10 before the Projects update (2026-09-25).</t>
   </si>
   <si>
     <t>Confirmed live on production 2026-09-23. The class has one learner, so the class figures follow that learner's.</t>
@@ -1170,7 +1170,7 @@
     <t>Learner "Learner User"</t>
   </si>
   <si>
-    <t>Practice Extra: Completed activities 4/4, above target 2/4, below target 0/4, 85%. Projects: Completed activities 0/5 (0 Gold medals, "-" average). Test: "This student has not activated the code yet".</t>
+    <t>Practice Extra: Completed activities 4/4, above target 2/4, below target 0/4, 85%. Projects: Completed activities 0/6 (0 Gold medals, "-" average). Test: "This student has not activated the code yet".</t>
   </si>
   <si>
     <t>Confirmed live on production 2026-09-23. The switch's checkbox is visually hidden — its label is clicked. From SOURCE toggleProgressBar / verifyTeacherAnalyticsBundleLevel.</t>

</xml_diff>